<commit_message>
feat(schedule): add trial solve impact preview
</commit_message>
<xml_diff>
--- a/datasets/real-school-furong/MASTER_DATA-v1.xlsx
+++ b/datasets/real-school-furong/MASTER_DATA-v1.xlsx
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MASTER_DATA v1；数据来源：2026-2027学年度上期芙蓉校区班级总课表；目标学期 2026-FALL-FR；17 个行政班、46 名教师、14 门课程、20 间教室、224 条教学需求；单双周轮换课程按第二位教师建模（该映射与真实课表零冲突）；普通课程绑定行政班教室，音乐、美术、科学课程使用可选教室池。</t>
+          <t>MASTER_DATA v1；数据来源：2026-2027学年度上期芙蓉校区班级总课表；目标学期 2026-FALL-FR；17 个行政班、46 名教师、14 门课程、20 间教室、224 条教学需求；单双周轮换课程按第二位教师建模（该映射与真实课表零冲突）；普通课程绑定行政班教室，音乐、美术、科学课程使用可选教室池；期望节次编码记录真实课表的原始排位，供 PREFER_ORIGINAL_SLOT 软规则贴原课表重排。</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K225"/>
+  <dimension ref="A1:L225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2772,6 +2772,7 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2830,6 +2831,11 @@
           <t>教室分配模式</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>期望节次编码</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2876,6 +2882,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>MON-1;TUE-2;DAY-4-2;DAY-5-3;DAY-5-4;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2922,6 +2933,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>TUE-1</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2968,6 +2984,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-2-3</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3014,6 +3035,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>DAY-4-1;MON-2;DAY-3-3;DAY-2-4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3060,6 +3086,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>DAY-5-1;DAY-1-3;DAY-4-3;DAY-3-4</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3106,6 +3137,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>DAY-3-2;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3152,6 +3188,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>DAY-5-2</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3198,6 +3239,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>DAY-1-4</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3244,6 +3290,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>DAY-4-4</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3290,6 +3341,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>DAY-1-5;DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3336,6 +3392,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>DAY-2-5</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3382,6 +3443,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3428,6 +3494,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>MON-1;TUE-1;DAY-4-2;DAY-5-2;DAY-5-3;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3474,6 +3545,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-5-1;MON-2;DAY-4-3</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3520,6 +3596,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>DAY-4-1;DAY-3-3</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3566,6 +3647,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>TUE-2</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3612,6 +3698,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>DAY-3-2;DAY-1-3;DAY-2-5;DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3658,6 +3749,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>DAY-2-3</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3704,6 +3800,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>DAY-1-4</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3750,6 +3851,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>DAY-2-4;DAY-5-4</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3796,6 +3902,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>DAY-3-4</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3842,6 +3953,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>DAY-4-4</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3888,6 +4004,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3934,6 +4055,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3980,6 +4106,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4026,6 +4157,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>MON-1;DAY-4-2;DAY-2-3;DAY-2-4;DAY-5-4;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4072,6 +4208,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>TUE-1;DAY-3-1;MON-2;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4118,6 +4259,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>DAY-4-1;TUE-2;DAY-3-2;DAY-1-4</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4164,6 +4310,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>DAY-5-1</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4210,6 +4361,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>DAY-5-2</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4256,6 +4412,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>DAY-1-3</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4302,6 +4463,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>DAY-3-3;DAY-4-4</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4348,6 +4514,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>DAY-4-3</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4394,6 +4565,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>DAY-5-3;DAY-2-5</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4440,6 +4616,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>DAY-3-4;DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4486,6 +4667,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4532,6 +4718,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4578,6 +4769,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>MON-1;TUE-1;DAY-4-3;DAY-4-4;DAY-5-4;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4624,6 +4820,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>DAY-3-1;MON-2;TUE-2;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4670,6 +4871,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>DAY-4-1;DAY-2-3;DAY-3-4;DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4716,6 +4922,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>DAY-5-1</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4762,6 +4973,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>DAY-3-2</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4808,6 +5024,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>DAY-4-2;DAY-3-3</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4854,6 +5075,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>DAY-5-2</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4900,6 +5126,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>DAY-1-3</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4946,6 +5177,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>DAY-5-3;DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4992,6 +5228,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>DAY-1-4;DAY-2-5</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5038,6 +5279,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>DAY-2-4</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5084,6 +5330,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5130,6 +5381,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>MON-1;TUE-1;DAY-4-2;DAY-5-3;DAY-5-4;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5176,6 +5432,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-2-4</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5222,6 +5483,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>DAY-4-1;DAY-5-1;DAY-1-3;DAY-3-4</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5268,6 +5534,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>MON-2;DAY-3-2;DAY-2-5;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5314,6 +5585,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>TUE-2</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5360,6 +5636,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>DAY-5-2;DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5406,6 +5687,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>DAY-2-3;DAY-4-4</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5452,6 +5738,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>DAY-3-3</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5498,6 +5789,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>DAY-4-3</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5544,6 +5840,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>DAY-1-4</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5590,6 +5891,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5636,6 +5942,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5682,6 +5993,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>MON-1;TUE-1;DAY-5-2;DAY-5-3;DAY-4-4;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5728,6 +6044,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-1-4;DAY-5-4;DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5774,6 +6095,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>DAY-4-1;DAY-5-1;MON-2;DAY-2-3</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5820,6 +6146,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>TUE-2</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5866,6 +6197,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>DAY-3-2</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5912,6 +6248,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>DAY-4-2</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5958,6 +6299,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>DAY-1-3</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6004,6 +6350,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>DAY-3-3</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6050,6 +6401,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>DAY-4-3;DAY-2-4</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6096,6 +6452,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>DAY-3-4;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6142,6 +6503,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6188,6 +6554,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>DAY-2-5</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6234,6 +6605,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6280,6 +6656,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>MON-1;DAY-4-1;DAY-5-1;TUE-2;DAY-4-4;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6326,6 +6707,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>TUE-1;DAY-5-3</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6372,6 +6758,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-1-3;DAY-2-4;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6418,6 +6809,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>MON-2</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6464,6 +6860,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>DAY-3-2</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6510,6 +6911,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>DAY-4-2;DAY-3-3</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6556,6 +6962,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>DAY-5-2;DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6602,6 +7013,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>DAY-2-3;DAY-4-3;DAY-5-4;DAY-1-6</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6648,6 +7064,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>DAY-1-4;DAY-5-6</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6694,6 +7115,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>DAY-3-4</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6740,6 +7166,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6786,6 +7217,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>DAY-2-5</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6832,6 +7268,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6878,6 +7319,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>DAY-3-6</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6924,6 +7370,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>DAY-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6970,6 +7421,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>MON-1;DAY-5-1;TUE-2;DAY-1-4;DAY-4-4;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7016,6 +7472,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>TUE-1;MON-2;DAY-3-2;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7062,6 +7523,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-2-4;DAY-4-5;DAY-1-6</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7108,6 +7574,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>DAY-4-1</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7154,6 +7625,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>DAY-4-2</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7200,6 +7676,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>DAY-5-2;DAY-1-3</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7246,6 +7727,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>DAY-2-3;DAY-5-3</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7292,6 +7778,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>DAY-3-3</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7338,6 +7829,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>DAY-4-3;DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7384,6 +7880,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>DAY-3-4;DAY-5-4</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7430,6 +7931,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>DAY-2-5;DAY-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7476,6 +7982,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7522,6 +8033,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>DAY-3-6</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7568,6 +8084,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>DAY-5-6</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7614,6 +8135,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>MON-1;TUE-1;DAY-4-1;DAY-5-2;DAY-3-5;DAY-3-6</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7660,6 +8186,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-2-4</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7706,6 +8237,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>DAY-5-1;TUE-2;DAY-1-3;DAY-3-3</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7752,6 +8288,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>MON-2;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7798,6 +8339,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>DAY-3-2</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7844,6 +8390,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>DAY-4-2;DAY-1-5;DAY-2-6;DAY-5-6</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -7890,6 +8441,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>DAY-2-3</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -7936,6 +8492,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>DAY-4-3</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -7982,6 +8543,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>DAY-5-3;DAY-4-4</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -8028,6 +8594,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>DAY-1-4</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8074,6 +8645,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>DAY-3-4</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8120,6 +8696,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>DAY-5-4;DAY-1-6</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8166,6 +8747,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>DAY-2-5;DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8212,6 +8798,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>DAY-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -8258,6 +8849,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>MON-1;TUE-1;DAY-5-2;DAY-5-3;DAY-4-4;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8304,6 +8900,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-5-1;MON-2;DAY-2-4</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8350,6 +8951,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>DAY-4-1;DAY-3-2</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -8396,6 +9002,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>TUE-2;DAY-4-3;DAY-5-4</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -8442,6 +9053,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>DAY-4-2;DAY-1-3;DAY-2-5;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -8488,6 +9104,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>DAY-2-3</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -8534,6 +9155,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>DAY-3-3;DAY-1-6</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -8580,6 +9206,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>DAY-1-4;DAY-3-4</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -8626,6 +9257,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -8672,6 +9308,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>DAY-4-5;DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -8718,6 +9359,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>DAY-3-6</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -8764,6 +9410,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>DAY-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -8810,6 +9461,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>DAY-5-6</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -8856,6 +9512,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>MON-1;DAY-4-1;DAY-5-2;DAY-2-4;DAY-5-4;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -8902,6 +9563,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>TUE-1;MON-2;DAY-3-3;DAY-4-3</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -8948,6 +9614,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -8994,6 +9665,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>DAY-5-1;DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -9040,6 +9716,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>TUE-2</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -9086,6 +9767,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>DAY-3-2</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -9132,6 +9818,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>DAY-4-2;DAY-5-3;DAY-3-6</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -9178,6 +9869,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>DAY-1-3;DAY-2-3;DAY-3-4;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -9224,6 +9920,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>DAY-1-4</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -9270,6 +9971,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>DAY-4-4;DAY-2-5</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -9316,6 +10022,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>DAY-1-6;DAY-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -9362,6 +10073,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -9408,6 +10124,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>DAY-5-6</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -9454,6 +10175,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>MON-1;TUE-1;DAY-4-1;TUE-2;DAY-5-3;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -9500,6 +10226,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-5-2;DAY-5-6</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -9546,6 +10277,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>DAY-5-1;DAY-4-2;DAY-2-3;DAY-3-3</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -9592,6 +10328,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>MON-2;DAY-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -9638,6 +10379,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>DAY-3-2;DAY-4-3;DAY-5-5;DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -9684,6 +10430,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>DAY-1-3;DAY-2-4</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -9730,6 +10481,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>DAY-1-4</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -9776,6 +10532,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>DAY-3-4;DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -9822,6 +10583,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>DAY-4-4</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -9868,6 +10634,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>DAY-5-4</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -9914,6 +10685,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>DAY-2-5</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -9960,6 +10736,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>DAY-4-5;DAY-1-6</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -10006,6 +10787,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>DAY-3-6</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -10052,6 +10838,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>MON-1;DAY-3-2;DAY-2-4;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -10098,6 +10889,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>TUE-1;DAY-4-1;MON-2;DAY-4-2;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -10144,6 +10940,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-1-4;DAY-2-5;DAY-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -10190,6 +10991,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>DAY-5-1</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -10236,6 +11042,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>TUE-2;DAY-3-3</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -10282,6 +11093,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>DAY-5-2</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -10328,6 +11144,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>DAY-1-3;DAY-2-3;DAY-3-4</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -10374,6 +11195,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>DAY-4-3;DAY-1-5;DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -10420,6 +11246,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>DAY-5-3</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -10466,6 +11297,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>DAY-4-4</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -10512,6 +11348,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>DAY-5-4</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -10558,6 +11399,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>DAY-4-5;DAY-5-6</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -10604,6 +11450,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>DAY-1-6</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -10650,6 +11501,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>DAY-3-6</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -10696,6 +11552,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>MON-1;DAY-4-1;DAY-5-2;DAY-2-3;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -10742,6 +11603,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>TUE-1;DAY-4-4;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -10788,6 +11654,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-4-3</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -10834,6 +11705,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>DAY-5-1;MON-2;DAY-3-2;DAY-2-4</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -10880,6 +11756,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>TUE-2;DAY-4-5;DAY-3-6;DAY-5-6</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -10926,6 +11807,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>DAY-4-2</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -10972,6 +11858,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>DAY-1-3</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -11018,6 +11909,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>DAY-3-3;DAY-1-4;DAY-2-5</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -11064,6 +11960,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>DAY-5-3;DAY-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -11110,6 +12011,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>DAY-3-4</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -11156,6 +12062,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>DAY-5-4</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -11202,6 +12113,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -11248,6 +12164,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>DAY-1-6</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -11294,6 +12215,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -11340,6 +12266,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>MON-1;TUE-1;DAY-4-1;DAY-5-2;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -11386,6 +12317,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-4-3;DAY-1-4;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -11432,6 +12368,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>DAY-5-1;DAY-1-6;DAY-3-6</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -11478,6 +12419,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>MON-2;DAY-3-4;DAY-5-6</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -11524,6 +12470,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>TUE-2;DAY-3-2</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -11570,6 +12521,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>DAY-4-2;DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -11616,6 +12572,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>DAY-1-3;DAY-3-3;DAY-2-4;DAY-4-4</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -11662,6 +12623,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>DAY-2-3</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -11708,6 +12674,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>DAY-5-3</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -11754,6 +12725,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>DAY-5-4</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -11800,6 +12776,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>DAY-2-5</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -11846,6 +12827,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -11892,6 +12878,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -11938,6 +12929,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>DAY-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -11984,6 +12980,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>MON-1;TUE-1;DAY-4-1;DAY-5-2;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -12030,6 +13031,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>DAY-3-1;TUE-2;DAY-4-2</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -12076,6 +13082,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>DAY-5-1;MON-2;DAY-3-2;DAY-2-4</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -12122,6 +13133,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>DAY-1-3;DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -12168,6 +13184,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>DAY-2-3</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -12214,6 +13235,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>DAY-3-3;DAY-5-3;DAY-1-4</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -12260,6 +13286,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>DAY-4-3</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -12306,6 +13337,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>DAY-3-4;DAY-4-4;DAY-2-5;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -12352,6 +13388,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>DAY-5-4;DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -12398,6 +13439,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -12444,6 +13490,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>DAY-1-6;DAY-5-6</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -12490,6 +13541,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>DAY-3-6</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -12536,6 +13592,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>DAY-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -12582,6 +13643,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>MON-1;TUE-1;DAY-5-1;DAY-4-2;DAY-3-5</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -12628,6 +13694,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>DAY-3-1;DAY-1-4;DAY-4-4;DAY-5-5</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -12674,6 +13745,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>DAY-4-1;DAY-3-2;DAY-1-3</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -12720,6 +13796,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>MON-2;DAY-4-3</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -12766,6 +13847,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>TUE-2;DAY-4-6</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -12812,6 +13898,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>DAY-5-2;DAY-2-4</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -12858,6 +13949,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>DAY-2-3;DAY-3-3;DAY-5-4;DAY-4-5</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -12904,6 +14000,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>DAY-5-3</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -12950,6 +14051,11 @@
           <t>FLEXIBLE</t>
         </is>
       </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>DAY-3-4;DAY-2-5;DAY-5-6</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -12996,6 +14102,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>DAY-1-5</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -13042,6 +14153,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>DAY-1-6</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -13088,6 +14204,11 @@
           <t>HOME</t>
         </is>
       </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>DAY-2-6</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -13132,6 +14253,11 @@
       <c r="K225" t="inlineStr">
         <is>
           <t>HOME</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>DAY-3-6</t>
         </is>
       </c>
     </row>

</xml_diff>